<commit_message>
Update access levels and add tabs to the roles and security spreadsheet
Refactor access level options from specific permissions to general tiers (Full Rights, Read & Write, View) and introduce "Tab" as an item type alongside "Form" and "Table" in the spreadsheet generation script.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: fdc1dbb1-98b8-4167-b03b-7dd1b42361c0
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6f7b72a6-6c9e-47f4-9b6c-14635073224d
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/scripts/exports/apps-roles-security-setup.xlsx
+++ b/scripts/exports/apps-roles-security-setup.xlsx
@@ -11,18 +11,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="117">
   <si>
     <t>Application Roles &amp; Security Setup — Permission Matrix</t>
   </si>
   <si>
-    <t>Access levels: Full (CRUD) = create/read/update/delete · Create/Edit = add &amp; modify · Edit Own = modify own records only · Read Only · No Access. Change any cell using its dropdown.</t>
+    <t>Permission levels: Full Rights = full control (create/read/update/delete &amp; settings) · Read &amp; Write = view and edit records · View = read-only access. Change any cell using its dropdown.</t>
   </si>
   <si>
     <t>PRODUCTION SHOP FLOOR</t>
   </si>
   <si>
-    <t>Form / Table</t>
+    <t>Form / Tab / Table</t>
   </si>
   <si>
     <t>Type</t>
@@ -46,6 +46,36 @@
     <t>Shop Floor Scheduler</t>
   </si>
   <si>
+    <t>Dashboard Tab</t>
+  </si>
+  <si>
+    <t>Tab</t>
+  </si>
+  <si>
+    <t>Overview of production status and KPIs</t>
+  </si>
+  <si>
+    <t>Full Rights</t>
+  </si>
+  <si>
+    <t>Read &amp; Write</t>
+  </si>
+  <si>
+    <t>View</t>
+  </si>
+  <si>
+    <t>Scheduling Tab</t>
+  </si>
+  <si>
+    <t>Production scheduling workspace</t>
+  </si>
+  <si>
+    <t>Reports Tab</t>
+  </si>
+  <si>
+    <t>Production, downtime, and quality reports</t>
+  </si>
+  <si>
     <t>Work Order Form</t>
   </si>
   <si>
@@ -55,15 +85,6 @@
     <t>Create and update production work orders</t>
   </si>
   <si>
-    <t>Full (CRUD)</t>
-  </si>
-  <si>
-    <t>Create/Edit</t>
-  </si>
-  <si>
-    <t>Read Only</t>
-  </si>
-  <si>
     <t>Production Schedule Form</t>
   </si>
   <si>
@@ -226,6 +247,21 @@
     <t>FIELD SERVICE CALENDAR</t>
   </si>
   <si>
+    <t>Calendar Tab</t>
+  </si>
+  <si>
+    <t>Main scheduling calendar view</t>
+  </si>
+  <si>
+    <t>Dispatch Board Tab</t>
+  </si>
+  <si>
+    <t>Assign and track technician jobs</t>
+  </si>
+  <si>
+    <t>Service performance and history reports</t>
+  </si>
+  <si>
     <t>Service Request Form</t>
   </si>
   <si>
@@ -254,9 +290,6 @@
   </si>
   <si>
     <t>Capture customer approval/signature</t>
-  </si>
-  <si>
-    <t>No Access</t>
   </si>
   <si>
     <t>Service Calendar Table</t>
@@ -380,7 +413,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -432,11 +465,6 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -465,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -507,9 +535,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -852,7 +877,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -942,11 +967,11 @@
       <c r="F6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>15</v>
+      <c r="G6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -991,14 +1016,14 @@
       <c r="E8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>15</v>
+      <c r="F8" s="10" t="s">
+        <v>16</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>15</v>
+      <c r="H8" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1006,10 +1031,10 @@
         <v>21</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>14</v>
@@ -1020,22 +1045,22 @@
       <c r="F9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>16</v>
+      <c r="G9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>14</v>
@@ -1043,25 +1068,25 @@
       <c r="E10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>15</v>
+      <c r="F10" s="10" t="s">
+        <v>16</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="9" t="s">
-        <v>15</v>
+      <c r="H10" s="8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>14</v>
@@ -1081,10 +1106,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>29</v>
@@ -1098,11 +1123,11 @@
       <c r="F12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>15</v>
+      <c r="G12" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1110,7 +1135,7 @@
         <v>30</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>31</v>
@@ -1121,14 +1146,14 @@
       <c r="E13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>16</v>
+      <c r="F13" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1136,7 +1161,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>33</v>
@@ -1147,14 +1172,14 @@
       <c r="E14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>14</v>
+      <c r="F14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1162,42 +1187,42 @@
         <v>34</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>16</v>
+      <c r="E15" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>16</v>
+      <c r="G15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>16</v>
+      <c r="E16" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="F16" s="10" t="s">
         <v>16</v>
@@ -1211,13 +1236,13 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>14</v>
@@ -1231,25 +1256,25 @@
       <c r="G17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="10" t="s">
-        <v>16</v>
+      <c r="H17" s="8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="9" t="s">
-        <v>15</v>
+      <c r="E18" s="10" t="s">
+        <v>16</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>16</v>
@@ -1257,661 +1282,808 @@
       <c r="G18" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
+      <c r="H18" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="17" t="s">
+      <c r="A21" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="18" t="s">
+      <c r="B21" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="D21" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="17" t="s">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18" t="s">
+      <c r="B24" s="16"/>
+      <c r="C24" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D25" s="17"/>
       <c r="E25" s="17"/>
       <c r="F25" s="18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G25" s="18"/>
       <c r="H25" s="18"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D26" s="17"/>
       <c r="E26" s="17"/>
       <c r="F26" s="18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G26" s="18"/>
       <c r="H26" s="18"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G27" s="18"/>
       <c r="H27" s="18"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
       <c r="F28" s="18" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="17" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D29" s="17"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G29" s="18"/>
       <c r="H29" s="18"/>
     </row>
-    <row r="32" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-    </row>
-    <row r="33" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+    </row>
+    <row r="36" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B36" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C36" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E36" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F36" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G36" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="H36" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B34" s="6" t="s">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H34" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B35" s="12" t="s">
+      <c r="C37" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G35" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B36" s="6" t="s">
+      <c r="C38" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H36" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G38" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="H38" s="19" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="11" t="s">
+      <c r="C39" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B39" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C39" s="13" t="s">
+      <c r="D39" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D39" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G39" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
+      <c r="B40" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C40" s="7" t="s">
+      <c r="D40" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D40" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H40" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="11" t="s">
+      <c r="B41" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C41" s="13" t="s">
+      <c r="D41" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D41" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G41" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="5" t="s">
+      <c r="B42" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C42" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C42" s="7" t="s">
+      <c r="D42" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D42" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G42" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H42" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
+      <c r="B43" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B43" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C43" s="13" t="s">
+      <c r="D43" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D43" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F43" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G43" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
+      <c r="B44" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C44" s="7" t="s">
+      <c r="D44" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D44" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G44" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H44" s="19" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
+      <c r="B45" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C45" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
+      <c r="D45" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G46" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B47" s="16"/>
-      <c r="C47" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
+      <c r="A47" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B48" s="5"/>
-      <c r="C48" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="G48" s="18"/>
-      <c r="H48" s="18"/>
+      <c r="A48" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C48" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B49" s="5"/>
-      <c r="C49" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G49" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="G49" s="18"/>
-      <c r="H49" s="18"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="5" t="s">
+      <c r="B53" s="16"/>
+      <c r="C53" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B50" s="5"/>
-      <c r="C50" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G50" s="18"/>
-      <c r="H50" s="18"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B51" s="5"/>
-      <c r="C51" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="G51" s="18"/>
-      <c r="H51" s="18"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52" s="5"/>
-      <c r="C52" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="G52" s="18"/>
-      <c r="H52" s="18"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B53" s="5"/>
-      <c r="C53" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="18" t="s">
-        <v>104</v>
-      </c>
-      <c r="G53" s="18"/>
-      <c r="H53" s="18"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="17" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="D54" s="17"/>
       <c r="E54" s="17"/>
       <c r="F54" s="18" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
       <c r="G54" s="18"/>
       <c r="H54" s="18"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B55" s="5"/>
       <c r="C55" s="17" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D55" s="17"/>
       <c r="E55" s="17"/>
       <c r="F55" s="18" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G55" s="18"/>
       <c r="H55" s="18"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="D56" s="17"/>
+      <c r="E56" s="17"/>
+      <c r="F56" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" s="5"/>
+      <c r="C57" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B58" s="5"/>
+      <c r="C58" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="D58" s="17"/>
+      <c r="E58" s="17"/>
+      <c r="F58" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B59" s="5"/>
+      <c r="C59" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="D59" s="17"/>
+      <c r="E59" s="17"/>
+      <c r="F59" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B60" s="5"/>
+      <c r="C60" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D60" s="17"/>
+      <c r="E60" s="17"/>
+      <c r="F60" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B61" s="5"/>
+      <c r="C61" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="58">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="F24:H24"/>
     <mergeCell ref="A25:B25"/>
@@ -1929,26 +2101,17 @@
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="C29:E29"/>
     <mergeCell ref="F29:H29"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A52:H52"/>
     <mergeCell ref="C53:E53"/>
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="A54:B54"/>
@@ -1957,16 +2120,34 @@
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="F55:H55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="F56:H56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="F61:H61"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid access level" error="Pick one of the access levels from the dropdown." sqref="D10:H18">
-      <formula1>"Full (CRUD),Create/Edit,Edit Own,Read Only,No Access"</formula1>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid access level" error="Pick one of the access levels from the dropdown." sqref="D10:H21">
+      <formula1>"Full Rights,Read &amp; Write,View"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid access level" error="Pick one of the access levels from the dropdown." sqref="D34:H44">
-      <formula1>"Full (CRUD),Create/Edit,Edit Own,Read Only,No Access"</formula1>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid access level" error="Pick one of the access levels from the dropdown." sqref="D37:H50">
+      <formula1>"Full Rights,Read &amp; Write,View"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid access level" error="Pick one of the access levels from the dropdown." sqref="D6:H18">
-      <formula1>"Full (CRUD),Create/Edit,Edit Own,Read Only,No Access"</formula1>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid access level" error="Pick one of the access levels from the dropdown." sqref="D6:H21">
+      <formula1>"Full Rights,Read &amp; Write,View"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>

</xml_diff>